<commit_message>
Split time and motion into Lagoons - Ibiza and Hills - Gems
Rebuilt from the updated QA/QC time + motion workbook, which adds Ibiza
T240 and T245, second sessions on several activities, and the roof and
Matterport rows T243 and T244 were missing. The header now reads
start 1 / end 1, which the parser accepts alongside start / end.

The default tab is now "Pilot time and motion Lagoons - Ibiza" with the
Ibiza units only; a new "Pilot time and motion Hills - Gems" tab carries
Gems-E511B. A tab lands on a page by its project prefix (SITES), and an
unknown prefix stops the build rather than dropping the unit.

Differences of 2 minutes or less between a row's minutes and its own
clock times are rounding and no longer flagged (ROUNDING).

The old activity log is renamed "Archived activities" and moves to the
last tab. On narrow screens the tabs wrap as one-line pills.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/qaqc-time-motion.xlsx
+++ b/data/qaqc-time-motion.xlsx
@@ -1,24 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackmwsmith/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackmwsmith/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB70C131-DC88-504B-82B6-DE01A9E7C574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8AA5C2-150B-7C46-902B-BF060CDD1986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="5" xr2:uid="{22CF0EF0-3217-9447-A544-6CCAFB8FCA32}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20500" activeTab="6" xr2:uid="{22CF0EF0-3217-9447-A544-6CCAFB8FCA32}"/>
   </bookViews>
   <sheets>
     <sheet name="Ibiza T241" sheetId="2" r:id="rId1"/>
     <sheet name="Ibiza T242" sheetId="3" r:id="rId2"/>
     <sheet name="Ibiza T243" sheetId="5" r:id="rId3"/>
     <sheet name="Ibiza T244" sheetId="6" r:id="rId4"/>
-    <sheet name="Gems-E511B" sheetId="1" r:id="rId5"/>
-    <sheet name="Gems-E511B_old" sheetId="4" r:id="rId6"/>
+    <sheet name="Ibiza T240" sheetId="7" r:id="rId5"/>
+    <sheet name="Ibiza T245" sheetId="8" r:id="rId6"/>
+    <sheet name="Gems-E511B" sheetId="1" r:id="rId7"/>
+    <sheet name="Gems-E511B_old" sheetId="4" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16442" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16484" uniqueCount="29">
   <si>
     <t>MEP general</t>
   </si>
@@ -119,6 +121,18 @@
   </si>
   <si>
     <t>total Matterport</t>
+  </si>
+  <si>
+    <t>start 1</t>
+  </si>
+  <si>
+    <t>end 1</t>
+  </si>
+  <si>
+    <t>start 2</t>
+  </si>
+  <si>
+    <t>end 2</t>
   </si>
 </sst>
 </file>
@@ -545,16 +559,16 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="E1" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="F1" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -627,13 +641,19 @@
         <v>16</v>
       </c>
       <c r="B6">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="C6">
         <v>1055</v>
       </c>
       <c r="D6">
         <v>1204</v>
+      </c>
+      <c r="E6">
+        <v>1456</v>
+      </c>
+      <c r="F6">
+        <v>1505</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -669,13 +689,13 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9">
-        <v>1112</v>
+        <v>1256</v>
       </c>
       <c r="D9">
-        <v>1120</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -712,7 +732,7 @@
       </c>
       <c r="B14">
         <f>B6</f>
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -730,7 +750,7 @@
       </c>
       <c r="B17">
         <f>B13+B14+B15</f>
-        <v>168</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -753,13 +773,17 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -825,7 +849,7 @@
         <v>16</v>
       </c>
       <c r="B6">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C6">
         <v>1450</v>
@@ -833,8 +857,14 @@
       <c r="D6">
         <v>1604</v>
       </c>
+      <c r="E6">
+        <v>1506</v>
+      </c>
+      <c r="F6">
+        <v>1512</v>
+      </c>
     </row>
-    <row r="7" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16384" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
@@ -848,7 +878,7 @@
         <v>1547</v>
       </c>
     </row>
-    <row r="8" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16384" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>20</v>
       </c>
@@ -49867,21 +49897,21 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16384" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B9">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C9">
-        <v>1547</v>
+        <v>1506</v>
       </c>
       <c r="D9">
-        <v>1604</v>
+        <v>1512</v>
       </c>
     </row>
-    <row r="10" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16384" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>19</v>
       </c>
@@ -49895,13 +49925,12 @@
         <v>1138</v>
       </c>
     </row>
-    <row r="11" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16384" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16384" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -49910,16 +49939,16 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16384" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
       <c r="B14">
         <f>B6</f>
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16384" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -49928,14 +49957,13 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:16384" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>21</v>
       </c>
       <c r="B17">
         <f>B13+B14+B15</f>
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -49945,27 +49973,32 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA35B3F3-D3D8-004D-BB48-8341B52BAC23}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1"/>
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B2">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C2">
         <v>957</v>
@@ -49973,13 +50006,28 @@
       <c r="D2">
         <v>1040</v>
       </c>
+      <c r="E2">
+        <v>1055</v>
+      </c>
+      <c r="F2">
+        <v>1112</v>
+      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="B3">
+        <v>17</v>
+      </c>
+      <c r="C3">
+        <v>1055</v>
+      </c>
+      <c r="D3">
+        <v>1112</v>
+      </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -49993,17 +50041,17 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B6">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="C6">
         <v>930</v>
@@ -50011,8 +50059,14 @@
       <c r="D6">
         <v>1019</v>
       </c>
+      <c r="E6">
+        <v>1515</v>
+      </c>
+      <c r="F6">
+        <v>1524</v>
+      </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
@@ -50026,7 +50080,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>20</v>
       </c>
@@ -50040,46 +50094,64 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>1515</v>
+      </c>
+      <c r="D9">
+        <v>1524</v>
+      </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>23</v>
       </c>
+      <c r="B10">
+        <v>88</v>
+      </c>
+      <c r="C10">
+        <v>1150</v>
+      </c>
+      <c r="D10">
+        <v>1318</v>
+      </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>9</v>
       </c>
       <c r="B13">
         <f>B2+B5</f>
-        <v>43</v>
+        <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
       <c r="B14">
         <f>B6</f>
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>24</v>
       </c>
       <c r="B15">
         <f>B10</f>
-        <v>0</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -50088,7 +50160,7 @@
       </c>
       <c r="B17">
         <f>B13+B14+B15</f>
-        <v>92</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -50098,27 +50170,32 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F71AD75-9824-2B41-B84C-64BDBF3E4EAE}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1"/>
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B2">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="C2">
         <v>1051</v>
@@ -50126,13 +50203,28 @@
       <c r="D2">
         <v>1134</v>
       </c>
+      <c r="E2">
+        <v>1113</v>
+      </c>
+      <c r="F2">
+        <v>1133</v>
+      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="B3">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>1113</v>
+      </c>
+      <c r="D3">
+        <v>1133</v>
+      </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -50146,17 +50238,17 @@
         <v>1134</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B6">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C6">
         <v>1045</v>
@@ -50164,8 +50256,14 @@
       <c r="D6">
         <v>1134</v>
       </c>
+      <c r="E6">
+        <v>1200</v>
+      </c>
+      <c r="F6">
+        <v>1214</v>
+      </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
@@ -50179,7 +50277,7 @@
         <v>1134</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>20</v>
       </c>
@@ -50193,46 +50291,64 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
+      <c r="B9">
+        <v>14</v>
+      </c>
+      <c r="C9">
+        <v>1200</v>
+      </c>
+      <c r="D9">
+        <v>1214</v>
+      </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>23</v>
       </c>
+      <c r="B10">
+        <v>90</v>
+      </c>
+      <c r="C10">
+        <v>1400</v>
+      </c>
+      <c r="D10">
+        <v>1530</v>
+      </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>9</v>
       </c>
       <c r="B13">
         <f>B2+B5</f>
-        <v>45</v>
+        <v>65</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
       <c r="B14">
         <f>B6</f>
-        <v>49</v>
+        <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>24</v>
       </c>
       <c r="B15">
         <f>B10</f>
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -50241,7 +50357,7 @@
       </c>
       <c r="B17">
         <f>B13+B14+B15</f>
-        <v>94</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -50250,6 +50366,354 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5E3B7AB-1F68-DE4A-AF3B-07083B85003A}">
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <v>50</v>
+      </c>
+      <c r="C2">
+        <v>945</v>
+      </c>
+      <c r="D2">
+        <v>1016</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1033</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>19</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1033</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>1033</v>
+      </c>
+      <c r="D4">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>68</v>
+      </c>
+      <c r="C6">
+        <v>1204</v>
+      </c>
+      <c r="D6">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>19</v>
+      </c>
+      <c r="C9">
+        <v>1215</v>
+      </c>
+      <c r="D9">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10">
+        <v>120</v>
+      </c>
+      <c r="C10">
+        <v>1530</v>
+      </c>
+      <c r="D10">
+        <v>1730</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13">
+        <f>B2+B5</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14">
+        <f>B6</f>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15">
+        <f>B10</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17">
+        <f>B13+B14+B15</f>
+        <v>238</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D99E7C1E-E34D-1A4F-A048-7FDBA65176E4}">
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <v>65</v>
+      </c>
+      <c r="C2">
+        <v>1421</v>
+      </c>
+      <c r="D2">
+        <v>1507</v>
+      </c>
+      <c r="E2">
+        <v>1134</v>
+      </c>
+      <c r="F2">
+        <v>1153</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>19</v>
+      </c>
+      <c r="C3">
+        <v>1134</v>
+      </c>
+      <c r="D3">
+        <v>1153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>62</v>
+      </c>
+      <c r="C6">
+        <v>1540</v>
+      </c>
+      <c r="D6">
+        <v>1621</v>
+      </c>
+      <c r="E6">
+        <v>1236</v>
+      </c>
+      <c r="F6">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>21</v>
+      </c>
+      <c r="C9">
+        <v>1236</v>
+      </c>
+      <c r="D9">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10">
+        <v>120</v>
+      </c>
+      <c r="C10">
+        <v>1730</v>
+      </c>
+      <c r="D10">
+        <v>1930</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13">
+        <f>B2+B5</f>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14">
+        <f>B6</f>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15">
+        <f>B10</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17">
+        <f>B13+B14+B15</f>
+        <v>247</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8E78D3C-2B2C-3041-89A1-9C61897F6A8E}">
   <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -50439,7 +50903,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DFA2DEA-ACE2-FC4B-9EF2-9D46EC3392BA}">
   <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Refresh time and motion from the latest workbook
Corrects T241 QA roof (14:56-15:05), T242 MEP roof (17m) and yard
(15:36-15:47, 11m), adds T240's second QA session, and sets Gems-E511B
tile tapping to 32m and QA functional to 4h 45m.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/qaqc-time-motion.xlsx
+++ b/data/qaqc-time-motion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackmwsmith/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8AA5C2-150B-7C46-902B-BF060CDD1986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D7E0A8-6787-2C43-8376-6C4D5C41C72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20500" activeTab="6" xr2:uid="{22CF0EF0-3217-9447-A544-6CCAFB8FCA32}"/>
   </bookViews>
@@ -692,10 +692,10 @@
         <v>9</v>
       </c>
       <c r="C9">
-        <v>1256</v>
+        <v>1456</v>
       </c>
       <c r="D9">
-        <v>1305</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -807,7 +807,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>1547</v>
@@ -821,13 +821,13 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C4">
-        <v>1451</v>
+        <v>1536</v>
       </c>
       <c r="D4">
-        <v>1459</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="5" spans="1:16384" x14ac:dyDescent="0.2">
@@ -50452,6 +50452,12 @@
       </c>
       <c r="D6">
         <v>1253</v>
+      </c>
+      <c r="E6">
+        <v>1215</v>
+      </c>
+      <c r="F6">
+        <v>1234</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -50791,7 +50797,7 @@
         <v>16</v>
       </c>
       <c r="B6">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="C6">
         <v>1029</v>
@@ -50813,7 +50819,7 @@
         <v>3</v>
       </c>
       <c r="B8">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="C8">
         <v>1422</v>
@@ -50870,7 +50876,7 @@
       </c>
       <c r="B14">
         <f>B6</f>
-        <v>275</v>
+        <v>285</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -50888,7 +50894,7 @@
       </c>
       <c r="B17">
         <f>B13+B14+B15</f>
-        <v>662</v>
+        <v>672</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Unit details and floor-area normalisation on time and motion
Floor area and bedrooms for Ibiza T240-T245 come from a new
data/time-motion-units.csv and show beside each unit's name. Each unit
card and the page summary gain recorded time per 100 m², and the
"Recorded time by unit" chart gets a Total time / Per 100 m² switch.

Also picks up the latest workbook, where Gems-E511B QA functional is
265 min and agrees with its clock times, and wraps the tab bar as
one-line pills below 960px, where four long tab names no longer fit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/qaqc-time-motion.xlsx
+++ b/data/qaqc-time-motion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackmwsmith/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D7E0A8-6787-2C43-8376-6C4D5C41C72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC4DF632-CD93-4345-B61C-ADE39239A3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20500" activeTab="6" xr2:uid="{22CF0EF0-3217-9447-A544-6CCAFB8FCA32}"/>
   </bookViews>
@@ -50542,6 +50542,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -50797,7 +50798,7 @@
         <v>16</v>
       </c>
       <c r="B6">
-        <v>285</v>
+        <v>265</v>
       </c>
       <c r="C6">
         <v>1029</v>
@@ -50876,7 +50877,7 @@
       </c>
       <c r="B14">
         <f>B6</f>
-        <v>285</v>
+        <v>265</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -50894,7 +50895,7 @@
       </c>
       <c r="B17">
         <f>B13+B14+B15</f>
-        <v>672</v>
+        <v>652</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>